<commit_message>
backtest update, looking to another restructuring
</commit_message>
<xml_diff>
--- a/config/Strategy.xlsx
+++ b/config/Strategy.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\htisec.local\HK Data\Department\PB\PB\Index Replication\index replicator\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50E9A9D4-1C22-44D9-92DD-022EA70D1F5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87395B24-9411-4E8B-AD38-1939819DDD02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -19,10 +19,19 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$K$1</definedName>
   </definedNames>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
       <xlwcv:version setVersion="1"/>
@@ -482,10 +491,10 @@
     <t>Strategy_CSI1000_QP</t>
   </si>
   <si>
-    <t>Strategy_CSI2000_LP</t>
-  </si>
-  <si>
     <t>SH932000</t>
+  </si>
+  <si>
+    <t>Strategy_CSI2000_QP</t>
   </si>
 </sst>
 </file>
@@ -896,7 +905,7 @@
     <col min="2" max="2" width="13.85546875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10.7109375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="19.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="20.5703125" customWidth="1"/>
+    <col min="5" max="5" width="25.28515625" customWidth="1"/>
     <col min="6" max="6" width="16.5703125" customWidth="1"/>
     <col min="7" max="7" width="23.5703125" bestFit="1" customWidth="1"/>
     <col min="8" max="9" width="23.5703125" customWidth="1"/>
@@ -991,7 +1000,7 @@
         <v>0</v>
       </c>
       <c r="C3" s="3">
-        <v>30000000</v>
+        <v>50000000</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>2</v>
@@ -1021,12 +1030,12 @@
       <c r="M3" s="4"/>
       <c r="N3" s="4"/>
     </row>
-    <row r="4" spans="1:14" ht="15.75" thickBot="1">
+    <row r="4" spans="1:14" ht="27" thickBot="1">
       <c r="A4" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B4" t="s">
         <v>36</v>
-      </c>
-      <c r="B4" t="s">
-        <v>37</v>
       </c>
       <c r="C4" s="3">
         <v>50000000</v>

</xml_diff>